<commit_message>
Update UBWC wrapper simulation flow
</commit_message>
<xml_diff>
--- a/docs/ubwc_reg_tables.xlsx
+++ b/docs/ubwc_reg_tables.xlsx
@@ -10,53 +10,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>模块</t>
+          <t>Module</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>寄存器地址</t>
+          <t>Register Address</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>寄存器名</t>
+          <t>Register Name</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>访问属性</t>
+          <t>Access</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>复位值</t>
+          <t>Reset Value</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>位段</t>
+          <t>Bit Field</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>字段名</t>
+          <t>Field Name</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>说明</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>备注</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -98,12 +98,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>IP版本号</t>
+          <t>IP version</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>固定返回32'h0001_0000</t>
+          <t>Returns fixed value 32'h0001_0000</t>
         </is>
       </c>
     </row>
@@ -145,12 +145,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>RTL日期</t>
+          <t>RTL date</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>固定返回32'h2026_0406</t>
+          <t>Returns fixed value 32'h2026_0406</t>
         </is>
       </c>
     </row>
@@ -192,12 +192,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>编码UBWC使能</t>
+          <t>Enable UBWC encoding</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>建议作为tile地址配置组最后写入; 写该寄存器会产生tile_addr_gen_cfg_vld脉冲</t>
+          <t>Recommended as the final write in the tile address configuration group</t>
         </is>
       </c>
     </row>
@@ -239,12 +239,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>一级bank swizzle使能</t>
+          <t>Level-1 bank swizzle enable</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>Same as above</t>
         </is>
       </c>
     </row>
@@ -286,12 +286,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>二级bank swizzle使能</t>
+          <t>Level-2 bank swizzle enable</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>Same as above</t>
         </is>
       </c>
     </row>
@@ -333,12 +333,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>三级bank swizzle使能</t>
+          <t>Level-3 bank swizzle enable</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>Same as above</t>
         </is>
       </c>
     </row>
@@ -380,12 +380,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>最高bank bit配置</t>
+          <t>Highest bank bit configuration</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>Same as above</t>
         </is>
       </c>
     </row>
@@ -427,12 +427,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>bank spread使能</t>
+          <t>Bank spread enable</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>Same as above</t>
         </is>
       </c>
     </row>
@@ -474,12 +474,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>4-line tile格式使能</t>
+          <t>4-line tile format enable</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>建议先写本寄存器再写REG_TILE_CFG0提交</t>
+          <t>Recommended to write this register before committing REG_TILE_CFG0</t>
         </is>
       </c>
     </row>
@@ -521,12 +521,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>RGBA 2:1 lossy格式选择</t>
+          <t>RGBA 2:1 lossy format select</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>Same as above</t>
         </is>
       </c>
     </row>
@@ -563,17 +563,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>pitch</t>
+          <t>tile_pitch</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>tile pitch配置</t>
+          <t>Tile pitch configuration</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>代码中实际有效位宽为11bit; o_pitch高位补0</t>
+          <t>The effective width in code is 11 bits</t>
         </is>
       </c>
     </row>
@@ -615,12 +615,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>编码CI输入类型</t>
+          <t>Encoded CI input type</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>建议作为CI配置组最后写入; 写该寄存器会产生o_enc_ci_vld脉冲</t>
+          <t>Recommended as the final write in the CI configuration group</t>
         </is>
       </c>
     </row>
@@ -662,12 +662,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>编码CI alen配置</t>
+          <t>Encoded CI alen configuration</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>Same as above</t>
         </is>
       </c>
     </row>
@@ -709,12 +709,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>编码CI格式</t>
+          <t>Encoded CI format</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>Same as above</t>
         </is>
       </c>
     </row>
@@ -751,17 +751,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>enc_ci_forced_pcm</t>
+          <t>reserved</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>强制PCM模式</t>
+          <t>Unused forced PCM configuration bit</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>Forced PCM is generated dynamically by the OTF path</t>
         </is>
       </c>
     </row>
@@ -803,12 +803,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>编码CI sideband配置</t>
+          <t>Encoded CI sideband configuration</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>位宽由SB_WIDTH参数决定</t>
+          <t>Width is determined by the SB_WIDTH parameter</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>编码CI lossy使能</t>
+          <t>Encoded CI lossy enable</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>UBWC CI配置0</t>
+          <t>UBWC CI configuration 0</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>UBWC CI配置1</t>
+          <t>UBWC CI configuration 1</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>UBWC CI配置2</t>
+          <t>UBWC CI configuration 2</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>UBWC CI配置3</t>
+          <t>UBWC CI configuration 3</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>UBWC CI配置4</t>
+          <t>UBWC CI configuration 4</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>UBWC CI配置5</t>
+          <t>UBWC CI configuration 5</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>UBWC CI配置6</t>
+          <t>UBWC CI configuration 6</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>UBWC CI配置7</t>
+          <t>UBWC CI configuration 7</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>UBWC CI配置8</t>
+          <t>UBWC CI configuration 8</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>UBWC CI配置9</t>
+          <t>UBWC CI configuration 9</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>UBWC CI配置10</t>
+          <t>UBWC CI configuration 10</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>UBWC CI配置11</t>
+          <t>UBWC CI configuration 11</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1461,12 +1461,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>输入OTF格式</t>
+          <t>Input OTF format</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>建议作为OTF配置组最后写入; 写该寄存器会产生o_otf_cfg_vld脉冲</t>
+          <t>Recommended as the final write in the OTF configuration group</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>输入图像宽度像素</t>
+          <t>Input image width in pixels</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>输入图像高度像素</t>
+          <t>Input image height in pixels</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>tile宽度像素</t>
+          <t>Tile width in pixels</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>tile高度像素</t>
+          <t>Tile height in pixels</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>A面tile列数</t>
+          <t>A-plane tile column count</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>B面tile列数</t>
+          <t>B-plane tile column count</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Y面压缩数据基地址低32位</t>
+          <t>Low 32 bits of the Y-plane compressed data base address</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -1837,12 +1837,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Y面压缩数据基地址高32位</t>
+          <t>High 32 bits of the Y-plane compressed data base address</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>AXI_AW=64时完整组成64bit地址</t>
+          <t>Forms the full 64-bit address when AXI_AW=64</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>UV或RGBA面压缩数据基地址低32位</t>
+          <t>Low 32 bits of the UV or RGBA-plane compressed data base address</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -1931,12 +1931,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>UV或RGBA面压缩数据基地址高32位</t>
+          <t>High 32 bits of the UV or RGBA-plane compressed data base address</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>AXI_AW=64时完整组成64bit地址</t>
+          <t>Forms the full 64-bit address when AXI_AW=64</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Y面metadata基地址低32位</t>
+          <t>Low 32 bits of the Y-plane metadata base address</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2025,12 +2025,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Y面metadata基地址高32位</t>
+          <t>High 32 bits of the Y-plane metadata base address</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>AXI_AW=64时完整组成64bit地址</t>
+          <t>Forms the full 64-bit address when AXI_AW=64</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>UV或RGBA面metadata基地址低32位</t>
+          <t>Low 32 bits of the UV or RGBA-plane metadata base address</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2119,12 +2119,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>UV或RGBA面metadata基地址高32位</t>
+          <t>High 32 bits of the UV or RGBA-plane metadata base address</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>AXI_AW=64时完整组成64bit地址</t>
+          <t>Forms the full 64-bit address when AXI_AW=64</t>
         </is>
       </c>
     </row>
@@ -2166,12 +2166,12 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>metadata有效区域宽度像素</t>
+          <t>Metadata active-area width in pixels</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>写0表示沿用整帧宽度</t>
+          <t>Writing 0 means using the full-frame width</t>
         </is>
       </c>
     </row>
@@ -2213,70 +2213,728 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>metadata有效区域高度像素</t>
+          <t>Metadata active-area height in pixels</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>写0表示沿用整帧高度</t>
+          <t>Writing 0 means using the full-frame height</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ubwc_enc_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>0x0054</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>REG_META_PITCH</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>0x00000000</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>31:0</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>meta_data_plane_pitch</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Metadata plane pitch in bytes</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Program this separately from the pixel-data pitch</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ubwc_enc_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>0x0058</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>REG_STATUS0</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>enc_idle</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Encoder core idle status</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ubwc_enc_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>0x0058</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>REG_STATUS0</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>enc_error</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Encoder core error status</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ubwc_enc_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>0x0058</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>REG_STATUS0</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>otf_to_tile_busy</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>OTF-to-tile busy status</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ubwc_enc_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>0x0058</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>REG_STATUS0</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>otf_to_tile_overflow</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>OTF-to-tile FIFO overflow status</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ubwc_enc_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>0x0058</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>REG_STATUS0</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>otf_err_bline</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>OTF input bad-line error status</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ubwc_enc_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>0x0058</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>REG_STATUS0</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>otf_err_bframe</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>OTF input bad-frame error status</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ubwc_enc_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>0x0058</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>REG_STATUS0</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>meta_err_0</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Metadata generator error 0 status</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Currently tied low</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ubwc_enc_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>0x0058</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>REG_STATUS0</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>meta_err_1</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Metadata generator error 1 status</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Currently tied low</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ubwc_enc_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>0x0058</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>REG_STATUS0</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>frame_done</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Encoder frame done status</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Live frame done input from wrapper</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ubwc_enc_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>0x005c</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>REG_STATUS1</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>7:0</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>stage_done</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Encoder stage done bitmap</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ubwc_enc_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>0x0060</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>REG_IRQ_CTRL</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>RW/W1P</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>0x00000001</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>irq_enable</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>IRQ enable</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Defaults to 1 after reset</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ubwc_enc_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>0x0060</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>REG_IRQ_CTRL</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>W1P</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>0x00000001</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>irq_clear</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>IRQ clear pulse</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Writing 1 generates an irq_clear pulse in the encoder clock domain; readback is 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ubwc_enc_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>0x0060</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>REG_IRQ_CTRL</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>irq_pending</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>IRQ pending status</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Synchronized into PCLK domain</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I47"/>
+  <autoFilter ref="A1:I61"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>模块</t>
+          <t>Module</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>寄存器地址</t>
+          <t>Register Address</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>寄存器名</t>
+          <t>Register Name</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>访问属性</t>
+          <t>Access</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>复位值</t>
+          <t>Reset Value</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>位段</t>
+          <t>Bit Field</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>字段名</t>
+          <t>Field Name</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>说明</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>备注</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -2318,12 +2976,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>IP版本号</t>
+          <t>IP version</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>固定返回32'h0001_0000</t>
+          <t>Returns fixed value 32'h0001_0000</t>
         </is>
       </c>
     </row>
@@ -2365,12 +3023,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>RTL日期</t>
+          <t>RTL date</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>固定返回32'h2026_0403</t>
+          <t>Returns fixed value 32'h2026_0403</t>
         </is>
       </c>
     </row>
@@ -2412,7 +3070,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>一级bank swizzle使能</t>
+          <t>Level-1 bank swizzle enable</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -2459,7 +3117,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>二级bank swizzle使能</t>
+          <t>Level-2 bank swizzle enable</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -2506,7 +3164,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>三级bank swizzle使能</t>
+          <t>Level-3 bank swizzle enable</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -2553,7 +3211,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>最高bank bit配置</t>
+          <t>Highest bank bit configuration</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -2600,7 +3258,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>bank spread使能</t>
+          <t>Bank spread enable</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -2647,7 +3305,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>4-line tile格式使能</t>
+          <t>4-line tile format enable</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -2694,7 +3352,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>RGBA 2:1 lossy格式选择</t>
+          <t>RGBA 2:1 lossy format select</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -2741,7 +3399,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>tile pitch配置</t>
+          <t>Tile pitch configuration</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -2788,7 +3446,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>CI输入类型</t>
+          <t>CI input type</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2835,12 +3493,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>CI sideband配置</t>
+          <t>CI sideband configuration</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>位宽由SB_WIDTH参数决定</t>
+          <t>Width is determined by the SB_WIDTH parameter</t>
         </is>
       </c>
     </row>
@@ -2882,7 +3540,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>CI lossy使能</t>
+          <t>CI lossy enable</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -2929,7 +3587,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>CI alpha mode配置</t>
+          <t>CI alpha mode configuration</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2976,12 +3634,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>ubwc_dec_vivo_top使能</t>
+          <t>ubwc_dec_vivo_top enable</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>复位后默认1</t>
+          <t>Defaults to 1 after reset</t>
         </is>
       </c>
     </row>
@@ -3023,12 +3681,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>vivo子模块软复位</t>
+          <t>VIVO submodule soft reset</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>可用于单独清空vivo内部状态</t>
+          <t>Can be used to independently clear VIVO internal state</t>
         </is>
       </c>
     </row>
@@ -3070,12 +3728,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>启动脉冲位</t>
+          <t>Start pulse bit</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>写1会翻转start toggle并在AXI域产生frame_start_pulse_axi; 读回固定为0; 建议最后写</t>
+          <t>Writing 1 toggles the start toggle and generates frame_start_pulse_axi in the AXI domain; readback is fixed to 0; recommended as the final write</t>
         </is>
       </c>
     </row>
@@ -3117,12 +3775,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>metadata/base格式配置</t>
+          <t>Metadata/base format configuration</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>通常与start在同一次写操作中一起下发</t>
+          <t>Usually issued with start in the same write</t>
         </is>
       </c>
     </row>
@@ -3159,12 +3817,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>meta_base_addr_rgba_uv[31:0]</t>
+          <t>meta_base_addr_rgba_y[31:0]</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>RGBA或UV metadata基地址低32位</t>
+          <t>Low 32 bits of the RGBA or Y metadata base address</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -3206,17 +3864,17 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>meta_base_addr_rgba_uv[63:32]</t>
+          <t>meta_base_addr_rgba_y[63:32]</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>RGBA或UV metadata基地址高32位</t>
+          <t>High 32 bits of the RGBA or Y metadata base address</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>AXI_AW=64时完整组成64bit地址</t>
+          <t>Forms the full 64-bit address when AXI_AW=64</t>
         </is>
       </c>
     </row>
@@ -3253,12 +3911,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>meta_base_addr_y[31:0]</t>
+          <t>meta_base_addr_uv[31:0]</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Y metadata基地址低32位</t>
+          <t>Low 32 bits of the UV metadata base address</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -3300,17 +3958,17 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>meta_base_addr_y[63:32]</t>
+          <t>meta_base_addr_uv[63:32]</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Y metadata基地址高32位</t>
+          <t>High 32 bits of the UV metadata base address</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>AXI_AW=64时完整组成64bit地址</t>
+          <t>Forms the full 64-bit address when AXI_AW=64</t>
         </is>
       </c>
     </row>
@@ -3352,7 +4010,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>metadata横向tile数量</t>
+          <t>Metadata tile count in the horizontal direction</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -3399,7 +4057,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>metadata纵向tile数量</t>
+          <t>Metadata tile count in the vertical direction</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -3446,7 +4104,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>输出图像有效宽度像素</t>
+          <t>Valid output image width in pixels</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -3493,7 +4151,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>输出OTF格式</t>
+          <t>Output OTF format</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3916,7 +4574,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>RGBA或UV tile基地址低32位</t>
+          <t>Low 32 bits of the RGBA or UV tile base address</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3963,12 +4621,12 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>RGBA或UV tile基地址高32位</t>
+          <t>High 32 bits of the RGBA or UV tile base address</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>AXI_AW=64时完整组成64bit地址</t>
+          <t>Forms the full 64-bit address when AXI_AW=64</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4668,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Y tile基地址低32位</t>
+          <t>Low 32 bits of the Y tile base address</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -4057,12 +4715,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Y tile基地址高32位</t>
+          <t>High 32 bits of the Y tile base address</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>AXI_AW=64时完整组成64bit地址</t>
+          <t>Forms the full 64-bit address when AXI_AW=64</t>
         </is>
       </c>
     </row>
@@ -4089,7 +4747,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>动态</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4104,12 +4762,12 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>当前帧是否处于active状态</t>
+          <t>Whether the current frame is active</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>启动后置1; 当前帧全部完成后清0</t>
+          <t>Set to 1 after start; cleared to 0 when the current frame fully completes</t>
         </is>
       </c>
     </row>
@@ -4136,7 +4794,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>动态</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4151,7 +4809,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>metadata读取阶段busy</t>
+          <t>Metadata read stage busy</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4183,7 +4841,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>动态</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -4198,7 +4856,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>tile读取阶段busy</t>
+          <t>Tile read stage busy</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4230,7 +4888,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>动态</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -4277,7 +4935,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>动态</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -4292,7 +4950,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>tile_to_otf阶段busy</t>
+          <t>tile_to_otf stage busy</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4324,7 +4982,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>动态</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -4339,12 +4997,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>当前所有busy输入均为0</t>
+          <t>All current busy inputs are 0</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>启动前和结束后都可能为1</t>
+          <t>May be 1 before start and after completion</t>
         </is>
       </c>
     </row>
@@ -4371,7 +5029,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>动态</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -4386,12 +5044,12 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>当前无busy且frame_active=0</t>
+          <t>No current busy and frame_active=0</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>建议与STATUS1[4]联合判断本帧结束</t>
+          <t>Recommended to combine with STATUS1[4] to judge frame completion</t>
         </is>
       </c>
     </row>
@@ -4433,12 +5091,12 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>metadata阶段已完成</t>
+          <t>Metadata stage completed</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>新一帧start时清零</t>
+          <t>Cleared when a new frame starts</t>
         </is>
       </c>
     </row>
@@ -4480,12 +5138,12 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>tile阶段已完成</t>
+          <t>Tile stage completed</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>新一帧start时清零</t>
+          <t>Cleared when a new frame starts</t>
         </is>
       </c>
     </row>
@@ -4527,12 +5185,12 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>vivo阶段已完成</t>
+          <t>VIVO stage completed</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>新一帧start时清零</t>
+          <t>Cleared when a new frame starts</t>
         </is>
       </c>
     </row>
@@ -4574,12 +5232,12 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>OTF输出阶段已完成</t>
+          <t>OTF output stage completed</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>新一帧start时清零</t>
+          <t>Cleared when a new frame starts</t>
         </is>
       </c>
     </row>
@@ -4621,12 +5279,12 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>整帧完成标志</t>
+          <t>Full-frame completion flag</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>最推荐的软件轮询位</t>
+          <t>Most recommended software polling bit</t>
         </is>
       </c>
     </row>
@@ -4668,12 +5326,12 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>本帧期间metadata阶段曾经进入busy</t>
+          <t>Metadata stage entered busy during this frame</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>用于避免未启动就误判done</t>
+          <t>Used to avoid falsely judging done before start</t>
         </is>
       </c>
     </row>
@@ -4715,12 +5373,12 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>本帧期间tile阶段曾经进入busy</t>
+          <t>Tile stage entered busy during this frame</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>Same as above</t>
         </is>
       </c>
     </row>
@@ -4762,12 +5420,12 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>本帧期间vivo阶段曾经进入busy</t>
+          <t>VIVO stage entered busy during this frame</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>Same as above</t>
         </is>
       </c>
     </row>
@@ -4809,17 +5467,252 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>本帧期间otf阶段曾经进入busy</t>
+          <t>OTF stage entered busy during this frame</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>同上</t>
+          <t>Same as above</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ubwc_dec_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>0x005c</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>APB_ADDR_STATUS2</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>6:0</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>vivo_idle_bits</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Raw ubwc_dec_vivo_top idle bitmap</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Passed through as o_idle[6:0] for software debug</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ubwc_dec_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>0x0060</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>APB_ADDR_STATUS3</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>6:0</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>vivo_error_bits</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Raw ubwc_dec_vivo_top error bitmap</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Passed through as o_error[6:0] for software debug</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ubwc_dec_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>0x0064</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>APB_ADDR_IRQ_CTRL</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>RW/W1P</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>0x00000001</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>irq_enable</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>IRQ enable</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Defaults to 1 after reset</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ubwc_dec_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>0x0064</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>APB_ADDR_IRQ_CTRL</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>W1P</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>0x00000001</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>irq_clear</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>IRQ clear pulse</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Writing 1 generates an irq_clear pulse in the AXI clock domain; readback is 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ubwc_dec_apb_reg_blk</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>0x0064</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>APB_ADDR_IRQ_CTRL</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>dynamic</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>irq_pending</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>IRQ pending status</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Synchronized into PCLK domain</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I55"/>
+  <autoFilter ref="A1:I60"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>